<commit_message>
feat(source): implement pending archive management with S3 integration for bulk uploads
</commit_message>
<xml_diff>
--- a/docs/lms_feature_list.xlsx
+++ b/docs/lms_feature_list.xlsx
@@ -8,19 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cluxssy/Code/phygitron360/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C742F182-4236-544A-A93B-098588A2BFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EC0CD6C-C62E-F042-9386-7967AD3B4FF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="19600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan (2)" sheetId="5" r:id="rId1"/>
-    <sheet name="Project Plan" sheetId="1" r:id="rId2"/>
-    <sheet name="Features" sheetId="2" r:id="rId3"/>
-    <sheet name="Summary" sheetId="3" r:id="rId4"/>
-    <sheet name="Employee Central Integration" sheetId="4" r:id="rId5"/>
+    <sheet name="Features" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" r:id="rId3"/>
+    <sheet name="Employee Central Integration" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Features!$A$4:$I$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Features!$A$4:$I$119</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="742">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1237" uniqueCount="742">
   <si>
     <t>EMPLOYEE CENTRAL (HRMS) &amp; LEARNING CENTRAL INTEGRATION MAP</t>
   </si>
@@ -2510,7 +2509,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -2570,22 +2569,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFCBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2765,9 +2753,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4241,238 +4226,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E60"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="39.1640625" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="75" customWidth="1"/>
-    <col min="4" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="63" t="s">
-        <v>38</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-    </row>
-    <row r="3" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="40" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="41" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="64" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-    </row>
-    <row r="5" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="52" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="52" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="53" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="47">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="52" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="53" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="47">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="52" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="53" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="52" t="s">
-        <v>46</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="47">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="52" t="s">
-        <v>46</v>
-      </c>
-      <c r="B10" s="53" t="s">
-        <v>77</v>
-      </c>
-      <c r="C10" s="47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="64" t="s">
-        <v>80</v>
-      </c>
-      <c r="B11" s="64"/>
-      <c r="C11" s="64"/>
-    </row>
-    <row r="12" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="54" t="s">
-        <v>81</v>
-      </c>
-      <c r="B12" s="57" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="44">
-        <v>1</v>
-      </c>
-      <c r="D12" s="64"/>
-    </row>
-    <row r="13" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="54" t="s">
-        <v>81</v>
-      </c>
-      <c r="B13" s="57" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="52" t="s">
-        <v>81</v>
-      </c>
-      <c r="B14" s="53" t="s">
-        <v>91</v>
-      </c>
-      <c r="C14" s="44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="52" t="s">
-        <v>81</v>
-      </c>
-      <c r="B15" s="53" t="s">
-        <v>104</v>
-      </c>
-      <c r="C15" s="44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="52" t="s">
-        <v>81</v>
-      </c>
-      <c r="B16" s="53" t="s">
-        <v>114</v>
-      </c>
-      <c r="C16" s="44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="58" t="s">
-        <v>118</v>
-      </c>
-      <c r="B17" s="48" t="s">
-        <v>119</v>
-      </c>
-      <c r="C17" s="51">
-        <f>SUM(C5:C10,C12:C16)</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="22" customHeight="1" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="20" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="21" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="23" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="24" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="25" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="26" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="27" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:3" ht="28" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="49" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="50" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="51" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="52" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="53" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="54" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="55" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="56" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="57" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="58" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="59" ht="22" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" ht="28" customHeight="1" x14ac:dyDescent="0.2"/>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -7888,7 +7641,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -8301,7 +8054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>